<commit_message>
analysis by city and month added
</commit_message>
<xml_diff>
--- a/Sales Report.xlsx
+++ b/Sales Report.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Sales_Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Product_Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="City_Performance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Monthly_Performance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -840,4 +842,316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Average Unit Price</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Orders Made</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Revenue Percentage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alexandria</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6625.246</v>
+      </c>
+      <c r="C2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D2" t="n">
+        <v>597478.6800000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" t="n">
+        <v>29.39440962138989</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2781.465555555556</v>
+      </c>
+      <c r="C3" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3" t="n">
+        <v>163075.65</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8.02290126130427</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Giza</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8515.562</v>
+      </c>
+      <c r="C4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>290831.27</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>14.30814816871632</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mansoura</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10459.949</v>
+      </c>
+      <c r="C5" t="n">
+        <v>52</v>
+      </c>
+      <c r="D5" t="n">
+        <v>352047.91</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>17.31984892397199</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tanta</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8792.45875</v>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="n">
+        <v>550698</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>27.09292085481639</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7849.54</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="n">
+        <v>78495.39999999999</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.861771169801151</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7287.049791666667</v>
+      </c>
+      <c r="C8" t="n">
+        <v>277</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2032626.91</v>
+      </c>
+      <c r="E8" t="n">
+        <v>48</v>
+      </c>
+      <c r="F8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Unit_Price</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Orders Made</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Revenue Percentage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7708.998076923077</v>
+      </c>
+      <c r="C2" t="n">
+        <v>153</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1109864.46</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>54.60246809386186</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6788.383636363636</v>
+      </c>
+      <c r="C3" t="n">
+        <v>124</v>
+      </c>
+      <c r="D3" t="n">
+        <v>922762.45</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F3" t="n">
+        <v>45.39753190613816</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7287.049791666667</v>
+      </c>
+      <c r="C4" t="n">
+        <v>277</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2032626.91</v>
+      </c>
+      <c r="E4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F4" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>